<commit_message>
feat: adiciona coluna criterio_atendido nos relatórios de gênero das 3 cidades
</commit_message>
<xml_diff>
--- a/resultados/maringa_oficial/relatorio_genero.xlsx
+++ b/resultados/maringa_oficial/relatorio_genero.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J285"/>
+  <dimension ref="A1:K285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,6 +476,11 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>criterio_atendido</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>caminho_relativo</t>
         </is>
       </c>
@@ -524,7 +529,8 @@
           <t>Arquivo geográfico DWG (AutoCAD) de bacias hidrográficas serializado como texto. Os termos 'man', 'men' e 'sex' são ruídos do formato binário DWG, não variáveis de gênero. Falso positivo técnico.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Bacias Hidrográficas 3ª Ordem - DWG.txt</t>
         </is>
@@ -574,7 +580,8 @@
           <t>Arquivo geográfico DWG (AutoCAD) de curvas de nível serializado como texto. Os termos 'man', 'men' e 'sex' são ruídos do formato binário DWG, não variáveis de gênero. Falso positivo técnico.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Curva de Nível (5m) - DWG.txt</t>
         </is>
@@ -624,7 +631,8 @@
           <t>O download retornou uma página HTML da Prefeitura de Maringá (redirecionamento de URL), não o arquivo de escala pretendido. Os termos 'mulher' e 'mulheres' foram encontrados em conteúdo editorial do site, não em dados estruturados.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\escala servidores abril 2026.txt</t>
         </is>
@@ -674,7 +682,8 @@
           <t>Mapa completo de Maringá em formato DWG (AutoCAD) serializado como texto. Os termos 'man', 'men' e 'sex' são ruídos do formato binário DWG, não variáveis de gênero. Falso positivo técnico.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Maringá - Completo (Mapa Janeiro_2025) - DWG.txt</t>
         </is>
@@ -724,7 +733,8 @@
           <t>Instalador de software SGS (Sistema de Gestão de Saneamento). Os termos 'man' e 'men' são referências técnicas do instalador (comandos ou metadados), sem relação com dados de gênero ou planejamento urbano. Falso positivo técnico.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Instalador SGS v12.6.txt</t>
         </is>
@@ -774,7 +784,8 @@
           <t>Lista de entidades cadastradas no CMDCA (Conselho Municipal dos Direitos da Criança e do Adolescente). O termo 'men' foi encontrado em nome de entidade registrada, não como variável de gênero estrutural nos dados. Falso positivo lexical.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\150425163658_listadasentidadescadastradasnocmdca_xls.xls</t>
         </is>
@@ -824,7 +835,8 @@
           <t>Ficha de notificação do SINAN para violência interpessoal e autoprovocada. Possui campos de gênero/sexo estruturais, mas trata-se de formulário vazio sem dados preenchidos, não constitui um dataset analisável. Documenta a intenção de coleta com recorte de gênero, mas não oferece dados para análise.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\1. Notificação de Violência Interpessoal Autoprovocada versão libreoffice_excel..xls</t>
         </is>
@@ -876,6 +888,11 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t>Pertinência Temática; Substantividade do Recorte; Apoio a Políticas Públicas</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>resultados\maringa_oficial\downloads\BANCO DE DADOS O-D MARINGÁ.xlsx</t>
         </is>
       </c>
@@ -906,10 +923,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>10</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2129863162- Thalisson Luiz Valduga Picinatto.zip</t>
         </is>
@@ -941,10 +962,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>14</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Planilha Monitoramento de Contatos.xls</t>
         </is>
@@ -976,10 +1001,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>5</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\PLANILHA CONTROLE ORÇAMENTÁRIO (LIBREOFFICE) - Baixar Arquivo.ods</t>
         </is>
@@ -1011,10 +1040,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>26</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\220623144437_modelopgrccplanilha__obras_nao_licenciaveis_xls.xls</t>
         </is>
@@ -1046,10 +1079,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
         <v>2</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Informações sobre vacinas disponíveis na UBS.xls</t>
         </is>
@@ -1081,10 +1118,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>7</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\- Modelo de Relatório de Competição - Entidades Esportivas.xlsx</t>
         </is>
@@ -1116,10 +1157,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
         <v>11</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\- Modelo de Relação de Ganhadores da Pesquisa de Preço.xls</t>
         </is>
@@ -1151,10 +1196,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
         <v>7</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\- Modelo de Relatório de Viagem - Entidades Esportivas.xlsx</t>
         </is>
@@ -1186,10 +1235,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
         <v>36</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Contagem Classificada 2022.xlsx</t>
         </is>
@@ -1221,10 +1274,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
         <v>4</v>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1905528587- Felipe Franco Tomazella.zip</t>
         </is>
@@ -1256,10 +1313,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
         <v>2</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Informações sobre medicamentos disponíveis na UBS.xls</t>
         </is>
@@ -1291,10 +1352,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
         <v>4</v>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\escala servidores abril 2026.xls</t>
         </is>
@@ -1326,10 +1391,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
         <v>67</v>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Contagem Classificada 2020.xlsx</t>
         </is>
@@ -1361,10 +1430,14 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="n">
         <v>4</v>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\escala servidores maio 2025.xls</t>
         </is>
@@ -1396,10 +1469,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
         <v>0</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Raquel Carreira.zip</t>
         </is>
@@ -1431,10 +1508,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="n">
         <v>0</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\RELATO PL 16457 - Selurb.txt</t>
         </is>
@@ -1466,10 +1547,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
         <v>0</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Relatório Projeto de Lei 16441-2022 Parque das Palmeiras.txt</t>
         </is>
@@ -1501,10 +1586,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
         <v>0</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Relatório Projeto de Lei 16449 - Parque José Bulla.txt</t>
         </is>
@@ -1536,10 +1625,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="n">
         <v>0</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Relatório Projeto de Lei 16451-2022 Cinquentenário.txt</t>
         </is>
@@ -1571,10 +1664,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
         <v>0</v>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Relatório Projeto de Lei 16469-2022 Alfredo Nyffeler.txt</t>
         </is>
@@ -1606,10 +1703,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="n">
         <v>0</v>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Renan Gustavo Parma dos Reis.zip</t>
         </is>
@@ -1641,10 +1742,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="n">
         <v>0</v>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\REPRESENTACAO_GRAFICA.zip</t>
         </is>
@@ -1676,10 +1781,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
         <v>0</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Resolução IAM n 02 de 30 de outubro de 2022 - REMESSA IAM.txt</t>
         </is>
@@ -1711,10 +1820,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
         <v>0</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Resolução nº 008_2025 - Autorização para Funcionamento da Educação Infantil da Escola Dom Bosco de Maringá.txt</t>
         </is>
@@ -1746,10 +1859,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
         <v>0</v>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Ribamar Nascimento - on-2023765901.zip</t>
         </is>
@@ -1781,10 +1898,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="n">
         <v>0</v>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Rubia Divino - on-1587878502.zip</t>
         </is>
@@ -1816,10 +1937,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="n">
         <v>0</v>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Soraya Ayumi Tory.zip</t>
         </is>
@@ -1851,10 +1976,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
         <v>0</v>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Thiago Ueda.zip</t>
         </is>
@@ -1886,10 +2015,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="n">
         <v>0</v>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Thiago Vinicius Alves Ueda - on-842160289.zip</t>
         </is>
@@ -1921,10 +2054,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="n">
         <v>0</v>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Vitoria Campanari - on-1528182808.zip</t>
         </is>
@@ -1956,10 +2093,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
         <v>0</v>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Comunicado aos Pais.txt</t>
         </is>
@@ -1991,10 +2132,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
         <v>0</v>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Comunicado de Paralisação de Atividades.txt</t>
         </is>
@@ -2026,10 +2171,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="n">
         <v>0</v>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Todos arquivos para reunião do dia 30_06_2022.zip</t>
         </is>
@@ -2061,10 +2210,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
         <v>0</v>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_ii__oficio_de_requerimento_do_cmdca_docx.docx.txt</t>
         </is>
@@ -2096,10 +2249,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="n">
         <v>0</v>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_iii__formulario_cadastral_docx.docx.txt</t>
         </is>
@@ -2131,10 +2288,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
         <v>0</v>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_iv__registro_fotografico_docx.docx.txt</t>
         </is>
@@ -2166,10 +2327,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="n">
         <v>0</v>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_ix___declaracao_de_escrituracao_contabi_docx.docx.txt</t>
         </is>
@@ -2201,10 +2366,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="n">
         <v>0</v>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_vi__declaracao_de_que_nao_incorrem_em_vedacoes_previstas_no_art__39_docx.docx.txt</t>
         </is>
@@ -2236,10 +2405,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="n">
         <v>0</v>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_vii__declaracao_de_capacidade_tecnica_e_operacional_docx.docx.txt</t>
         </is>
@@ -2271,10 +2444,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="n">
         <v>0</v>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_viii___declaracao_de_que_nao_serao_remunerados_membros_do_poder_publico__docx.docx.txt</t>
         </is>
@@ -2306,10 +2483,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="n">
         <v>0</v>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_x__declaracao_da_nao_ocorrencia_de_impedimentos_docx.docx.txt</t>
         </is>
@@ -2341,10 +2522,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="n">
         <v>0</v>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_xi__declaracao_de_nao_existencia_de_trabalhadores_menores_docx.docx.txt</t>
         </is>
@@ -2376,10 +2561,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="n">
         <v>0</v>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_xii__declaracao_de_idoneidade_docx.docx.txt</t>
         </is>
@@ -2411,10 +2600,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="n">
         <v>0</v>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_xiii_relacao_nominal_dos_dirigentes_docx.docx.txt</t>
         </is>
@@ -2446,10 +2639,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="n">
         <v>0</v>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\060825101704_anexo_xiv_relatorio_de_atividades_docx.docx.txt</t>
         </is>
@@ -2481,10 +2678,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
         <v>0</v>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\William Farias - on-808283414.zip</t>
         </is>
@@ -2516,10 +2717,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="n">
         <v>0</v>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Enne Flicts Dias Pedroza.zip</t>
         </is>
@@ -2551,10 +2756,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="n">
         <v>0</v>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Erica Paiva.zip</t>
         </is>
@@ -2586,10 +2795,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="n">
         <v>0</v>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\escala servidores julho 2025.txt</t>
         </is>
@@ -2621,10 +2834,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="n">
         <v>0</v>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Eva Alves Lacerda - on-1962680317.zip</t>
         </is>
@@ -2656,10 +2873,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="n">
         <v>0</v>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Bairros (19_01_2026).zip</t>
         </is>
@@ -2691,10 +2912,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="n">
         <v>0</v>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Baixar arquivo.zip</t>
         </is>
@@ -2726,10 +2951,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="n">
         <v>0</v>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Bruno Arnold Pesch - on-2028299148.zip</t>
         </is>
@@ -2761,10 +2990,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="n">
         <v>0</v>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Bruno Arnold Pesch.zip</t>
         </is>
@@ -2796,10 +3029,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" t="n">
         <v>0</v>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Bruno Rosa - on-1233333133.zip</t>
         </is>
@@ -2831,10 +3068,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" t="n">
         <v>0</v>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Camila Carmona Sabater - on-437398068.zip</t>
         </is>
@@ -2866,10 +3107,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
         <v>0</v>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Camila Fernanda Silva de Souza - on-818302109.zip</t>
         </is>
@@ -2901,10 +3146,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
         <v>0</v>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Camila Lozeckyi.zip</t>
         </is>
@@ -2936,10 +3185,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" t="n">
         <v>0</v>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Cardápio Restaurantes Populares Janeiro 2026.txt</t>
         </is>
@@ -2971,10 +3224,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" t="n">
         <v>0</v>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\070823161515_spcv_s_a_xlsx.xlsx.txt</t>
         </is>
@@ -3006,10 +3263,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F70" t="inlineStr"/>
       <c r="G70" t="n">
         <v>0</v>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\certificados_inmetro-20260514_1.zip</t>
         </is>
@@ -3041,10 +3302,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F71" t="inlineStr"/>
       <c r="G71" t="n">
         <v>0</v>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\cfaa045ef96b.docx.txt</t>
         </is>
@@ -3076,10 +3341,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="n">
         <v>0</v>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Gabriel Silva Batista.zip</t>
         </is>
@@ -3111,10 +3380,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr"/>
       <c r="G73" t="n">
         <v>0</v>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Gabriela Tornai.zip</t>
         </is>
@@ -3146,10 +3419,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" t="n">
         <v>0</v>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Geórgia Kimura Noda - on-1034055903.zip</t>
         </is>
@@ -3181,10 +3458,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F75" t="inlineStr"/>
       <c r="G75" t="n">
         <v>0</v>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Guilherme de Souza Oliveira.zip</t>
         </is>
@@ -3216,10 +3497,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr"/>
       <c r="G76" t="n">
         <v>0</v>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Guilherme Veneral Barbosa.zip</t>
         </is>
@@ -3251,10 +3536,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" t="n">
         <v>0</v>
       </c>
-      <c r="J77" t="inlineStr">
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Hidrografia (19_01_2026).zip</t>
         </is>
@@ -3286,10 +3575,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F78" t="inlineStr"/>
       <c r="G78" t="n">
         <v>0</v>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Ieda Marinho de Sousa - on-1703172706.zip</t>
         </is>
@@ -3321,10 +3614,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr"/>
       <c r="G79" t="n">
         <v>0</v>
       </c>
-      <c r="J79" t="inlineStr">
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Igor Gustavo Pereira Gilberto.zip</t>
         </is>
@@ -3356,10 +3653,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F80" t="inlineStr"/>
       <c r="G80" t="n">
         <v>0</v>
       </c>
-      <c r="J80" t="inlineStr">
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Informações sobre medicamentos disponíveis na UBS.txt</t>
         </is>
@@ -3391,10 +3692,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="n">
         <v>0</v>
       </c>
-      <c r="J81" t="inlineStr">
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Convite + ficha + publicação DOM_2022.txt</t>
         </is>
@@ -3426,10 +3731,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F82" t="inlineStr"/>
       <c r="G82" t="n">
         <v>0</v>
       </c>
-      <c r="J82" t="inlineStr">
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\César Augusto Ferreira Santos Silva - on-761403699.zip</t>
         </is>
@@ -3461,10 +3770,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr"/>
       <c r="G83" t="n">
         <v>0</v>
       </c>
-      <c r="J83" t="inlineStr">
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Diretriz viária (19_01_2026).zip</t>
         </is>
@@ -3496,10 +3809,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" t="n">
         <v>0</v>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Douglas Kodi Seto Takeguma - on-2022187766.zip</t>
         </is>
@@ -3531,10 +3848,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F85" t="inlineStr"/>
       <c r="G85" t="n">
         <v>0</v>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Douglas Kodi Seto Takeguma.zip</t>
         </is>
@@ -3566,10 +3887,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F86" t="inlineStr"/>
       <c r="G86" t="n">
         <v>0</v>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Edipo Leandro Ferreira - on-1532456533.zip</t>
         </is>
@@ -3601,10 +3926,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" t="n">
         <v>0</v>
       </c>
-      <c r="J87" t="inlineStr">
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Elisa Riemer - on-622529863.zip</t>
         </is>
@@ -3636,10 +3965,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F88" t="inlineStr"/>
       <c r="G88" t="n">
         <v>0</v>
       </c>
-      <c r="J88" t="inlineStr">
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Laiana Moraes de Azevedo.zip</t>
         </is>
@@ -3671,10 +4004,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="n">
         <v>0</v>
       </c>
-      <c r="J89" t="inlineStr">
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Laís Azevedo Fialho - on-1404712152.zip</t>
         </is>
@@ -3706,10 +4043,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr"/>
       <c r="G90" t="n">
         <v>0</v>
       </c>
-      <c r="J90" t="inlineStr">
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Lei uso e ocupação (19_01_2026).zip</t>
         </is>
@@ -3741,10 +4082,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" t="n">
         <v>0</v>
       </c>
-      <c r="J91" t="inlineStr">
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Leonardo Vinicius Fabiano - on-1408453596.zip</t>
         </is>
@@ -3776,10 +4121,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" t="n">
         <v>0</v>
       </c>
-      <c r="J92" t="inlineStr">
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Leonardo Vinicius Fabiano.zip</t>
         </is>
@@ -3811,10 +4160,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" t="n">
         <v>0</v>
       </c>
-      <c r="J93" t="inlineStr">
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Lirian Lopes - on-330333178.zip</t>
         </is>
@@ -3846,10 +4199,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F94" t="inlineStr"/>
       <c r="G94" t="n">
         <v>0</v>
       </c>
-      <c r="J94" t="inlineStr">
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Logradouros (19_01_2026).zip</t>
         </is>
@@ -3881,10 +4238,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="n">
         <v>0</v>
       </c>
-      <c r="J95" t="inlineStr">
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Lote rural (19_01_2026).zip</t>
         </is>
@@ -3916,10 +4277,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F96" t="inlineStr"/>
       <c r="G96" t="n">
         <v>0</v>
       </c>
-      <c r="J96" t="inlineStr">
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Lotes (19_01_2026).zip</t>
         </is>
@@ -3951,10 +4316,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" t="n">
         <v>0</v>
       </c>
-      <c r="J97" t="inlineStr">
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\f01fb161a82c.docx.txt</t>
         </is>
@@ -3986,10 +4355,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="n">
         <v>0</v>
       </c>
-      <c r="J98" t="inlineStr">
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Felipe Cosmos de Oliveira - on-362163241.zip</t>
         </is>
@@ -4021,10 +4394,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" t="n">
         <v>0</v>
       </c>
-      <c r="J99" t="inlineStr">
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Felipe de Moraes (Momo) - on-1006308251.zip</t>
         </is>
@@ -4056,10 +4433,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="n">
         <v>0</v>
       </c>
-      <c r="J100" t="inlineStr">
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Felipe Franco da Costa ( Dj Maré) - on-1019756110.zip</t>
         </is>
@@ -4091,10 +4472,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F101" t="inlineStr"/>
       <c r="G101" t="n">
         <v>0</v>
       </c>
-      <c r="J101" t="inlineStr">
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Felipe Index - on-316499473.zip</t>
         </is>
@@ -4126,10 +4511,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" t="n">
         <v>0</v>
       </c>
-      <c r="J102" t="inlineStr">
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Fernando Ponce.zip</t>
         </is>
@@ -4161,10 +4550,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" t="n">
         <v>0</v>
       </c>
-      <c r="J103" t="inlineStr">
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Formulário de Registro de Produtos Produzidos.txt</t>
         </is>
@@ -4196,10 +4589,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F104" t="inlineStr"/>
       <c r="G104" t="n">
         <v>0</v>
       </c>
-      <c r="J104" t="inlineStr">
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Luisa Peralta Krauze - on-1378490753.zip</t>
         </is>
@@ -4231,10 +4628,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="n">
         <v>0</v>
       </c>
-      <c r="J105" t="inlineStr">
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Macrozoneamento (19_01_2026).zip</t>
         </is>
@@ -4266,10 +4667,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F106" t="inlineStr"/>
       <c r="G106" t="n">
         <v>0</v>
       </c>
-      <c r="J106" t="inlineStr">
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Marcelo Yukio Goto - on-380783380.zip</t>
         </is>
@@ -4301,10 +4706,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F107" t="inlineStr"/>
       <c r="G107" t="n">
         <v>0</v>
       </c>
-      <c r="J107" t="inlineStr">
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Matheus Navarro Pedroso - on-1344236872.zip</t>
         </is>
@@ -4336,10 +4745,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F108" t="inlineStr"/>
       <c r="G108" t="n">
         <v>0</v>
       </c>
-      <c r="J108" t="inlineStr">
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\MESTRE CHUPPIM - on-1622808830.zip</t>
         </is>
@@ -4371,10 +4784,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="n">
         <v>0</v>
       </c>
-      <c r="J109" t="inlineStr">
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Michelle Cerqueira César Tambosi - on-2041072367.zip</t>
         </is>
@@ -4406,10 +4823,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F110" t="inlineStr"/>
       <c r="G110" t="n">
         <v>0</v>
       </c>
-      <c r="J110" t="inlineStr">
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Michelly cristina de oliveira - on-1737886068.zip</t>
         </is>
@@ -4441,10 +4862,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F111" t="inlineStr"/>
       <c r="G111" t="n">
         <v>0</v>
       </c>
-      <c r="J111" t="inlineStr">
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Milena Plahtyn Fernandes.zip</t>
         </is>
@@ -4476,10 +4901,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F112" t="inlineStr"/>
       <c r="G112" t="n">
         <v>0</v>
       </c>
-      <c r="J112" t="inlineStr">
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\MINUTA ATA 7ª REUNIÃO ORDINÁRIA.txt</t>
         </is>
@@ -4511,10 +4940,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F113" t="inlineStr"/>
       <c r="G113" t="n">
         <v>0</v>
       </c>
-      <c r="J113" t="inlineStr">
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Nayara Araujo.zip</t>
         </is>
@@ -4546,10 +4979,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F114" t="inlineStr"/>
       <c r="G114" t="n">
         <v>0</v>
       </c>
-      <c r="J114" t="inlineStr">
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Néia Silva Pereira Trindade.zip</t>
         </is>
@@ -4581,10 +5018,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F115" t="inlineStr"/>
       <c r="G115" t="n">
         <v>0</v>
       </c>
-      <c r="J115" t="inlineStr">
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1022497569- Nagela Terezinha de Souza.zip</t>
         </is>
@@ -4616,10 +5057,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F116" t="inlineStr"/>
       <c r="G116" t="n">
         <v>0</v>
       </c>
-      <c r="J116" t="inlineStr">
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Jaqueline Silva do Nascimento.zip</t>
         </is>
@@ -4651,10 +5096,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F117" t="inlineStr"/>
       <c r="G117" t="n">
         <v>0</v>
       </c>
-      <c r="J117" t="inlineStr">
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\JEAN MICHEL - on-1729307989.zip</t>
         </is>
@@ -4686,10 +5135,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F118" t="inlineStr"/>
       <c r="G118" t="n">
         <v>0</v>
       </c>
-      <c r="J118" t="inlineStr">
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\João Gabriel Kowalski - on-241195902.zip</t>
         </is>
@@ -4721,10 +5174,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F119" t="inlineStr"/>
       <c r="G119" t="n">
         <v>0</v>
       </c>
-      <c r="J119" t="inlineStr">
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\KÊNIA BRITO BERGO.zip</t>
         </is>
@@ -4756,10 +5213,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F120" t="inlineStr"/>
       <c r="G120" t="n">
         <v>0</v>
       </c>
-      <c r="J120" t="inlineStr">
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1065356688-Associação de Capoeira Centro Cultural Sucena.zip</t>
         </is>
@@ -4791,10 +5252,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="n">
         <v>0</v>
       </c>
-      <c r="J121" t="inlineStr">
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1071675793- Arena das Artes.zip</t>
         </is>
@@ -4826,10 +5291,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F122" t="inlineStr"/>
       <c r="G122" t="n">
         <v>0</v>
       </c>
-      <c r="J122" t="inlineStr">
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1120302651- Alexandre Penha.zip</t>
         </is>
@@ -4861,10 +5330,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F123" t="inlineStr"/>
       <c r="G123" t="n">
         <v>0</v>
       </c>
-      <c r="J123" t="inlineStr">
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1146440847-Mateus Moscheta.zip</t>
         </is>
@@ -4896,10 +5369,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F124" t="inlineStr"/>
       <c r="G124" t="n">
         <v>0</v>
       </c>
-      <c r="J124" t="inlineStr">
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1183133970- Nayara Araujo.zip</t>
         </is>
@@ -4931,10 +5408,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F125" t="inlineStr"/>
       <c r="G125" t="n">
         <v>0</v>
       </c>
-      <c r="J125" t="inlineStr">
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1203309085-Renan Gustavo Parma dos Reis.zip</t>
         </is>
@@ -4966,10 +5447,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F126" t="inlineStr"/>
       <c r="G126" t="n">
         <v>0</v>
       </c>
-      <c r="J126" t="inlineStr">
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1213542027-LILIAN FLÁVIA OJEIKA AVANZÍ.zip</t>
         </is>
@@ -5001,10 +5486,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F127" t="inlineStr"/>
       <c r="G127" t="n">
         <v>0</v>
       </c>
-      <c r="J127" t="inlineStr">
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1215659232- Leonardo Vinicius Fabiano.zip</t>
         </is>
@@ -5036,10 +5525,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F128" t="inlineStr"/>
       <c r="G128" t="n">
         <v>0</v>
       </c>
-      <c r="J128" t="inlineStr">
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1223311064-CASA LUANDA ASSOCIAÇÃO AFRO-CULTURAL.zip</t>
         </is>
@@ -5071,10 +5564,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" t="n">
         <v>0</v>
       </c>
-      <c r="J129" t="inlineStr">
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1225272911- Ana Clara Poltronieri Borges.zip</t>
         </is>
@@ -5106,10 +5603,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F130" t="inlineStr"/>
       <c r="G130" t="n">
         <v>0</v>
       </c>
-      <c r="J130" t="inlineStr">
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1239836778- Érica Paiva Rosa.zip</t>
         </is>
@@ -5141,10 +5642,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="n">
         <v>0</v>
       </c>
-      <c r="J131" t="inlineStr">
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1254825343-LEONARDO VINICIUS FABIANO.zip</t>
         </is>
@@ -5176,10 +5681,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F132" t="inlineStr"/>
       <c r="G132" t="n">
         <v>0</v>
       </c>
-      <c r="J132" t="inlineStr">
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1300640591- Mateus Moscheta.zip</t>
         </is>
@@ -5211,10 +5720,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F133" t="inlineStr"/>
       <c r="G133" t="n">
         <v>0</v>
       </c>
-      <c r="J133" t="inlineStr">
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Lucas Fiorindo - on-2010728686.zip</t>
         </is>
@@ -5246,10 +5759,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F134" t="inlineStr"/>
       <c r="G134" t="n">
         <v>0</v>
       </c>
-      <c r="J134" t="inlineStr">
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Lucas Fiorindo.zip</t>
         </is>
@@ -5281,10 +5798,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F135" t="inlineStr"/>
       <c r="G135" t="n">
         <v>0</v>
       </c>
-      <c r="J135" t="inlineStr">
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Ludmila de Almeida Castanheira - on-1968990312.zip</t>
         </is>
@@ -5316,10 +5837,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F136" t="inlineStr"/>
       <c r="G136" t="n">
         <v>0</v>
       </c>
-      <c r="J136" t="inlineStr">
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1352104052- Érica Paiva Rosa.zip</t>
         </is>
@@ -5351,10 +5876,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F137" t="inlineStr"/>
       <c r="G137" t="n">
         <v>0</v>
       </c>
-      <c r="J137" t="inlineStr">
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1378030105- Bianca Ribeiro.zip</t>
         </is>
@@ -5386,10 +5915,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F138" t="inlineStr"/>
       <c r="G138" t="n">
         <v>0</v>
       </c>
-      <c r="J138" t="inlineStr">
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1421693279- Thais Andressa Arantes Couto.zip</t>
         </is>
@@ -5421,10 +5954,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F139" t="inlineStr"/>
       <c r="G139" t="n">
         <v>0</v>
       </c>
-      <c r="J139" t="inlineStr">
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1422858460- Vitoria Campanari.zip</t>
         </is>
@@ -5456,10 +5993,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F140" t="inlineStr"/>
       <c r="G140" t="n">
         <v>0</v>
       </c>
-      <c r="J140" t="inlineStr">
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1457672720- Piera Paula Schnaider do Nascimento.zip</t>
         </is>
@@ -5491,10 +6032,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F141" t="inlineStr"/>
       <c r="G141" t="n">
         <v>0</v>
       </c>
-      <c r="J141" t="inlineStr">
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1501048750-Nayara Tamires Correia de Araujo.zip</t>
         </is>
@@ -5526,10 +6071,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F142" t="inlineStr"/>
       <c r="G142" t="n">
         <v>0</v>
       </c>
-      <c r="J142" t="inlineStr">
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1509163372-LUCAS FIORINDO.zip</t>
         </is>
@@ -5561,10 +6110,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F143" t="inlineStr"/>
       <c r="G143" t="n">
         <v>0</v>
       </c>
-      <c r="J143" t="inlineStr">
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1514962176- Aline Amenencia de Souza.zip</t>
         </is>
@@ -5596,10 +6149,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F144" t="inlineStr"/>
       <c r="G144" t="n">
         <v>0</v>
       </c>
-      <c r="J144" t="inlineStr">
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1529968768-MARIELA LAMBERTI DE ABREU.zip</t>
         </is>
@@ -5631,10 +6188,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F145" t="inlineStr"/>
       <c r="G145" t="n">
         <v>0</v>
       </c>
-      <c r="J145" t="inlineStr">
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1530423972-Vitoria Campanari.zip</t>
         </is>
@@ -5666,10 +6227,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F146" t="inlineStr"/>
       <c r="G146" t="n">
         <v>0</v>
       </c>
-      <c r="J146" t="inlineStr">
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1536623014- João Paulo Baliscei.zip</t>
         </is>
@@ -5701,10 +6266,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F147" t="inlineStr"/>
       <c r="G147" t="n">
         <v>0</v>
       </c>
-      <c r="J147" t="inlineStr">
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1542656743- Joice Bianca Gomes.zip</t>
         </is>
@@ -5736,10 +6305,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F148" t="inlineStr"/>
       <c r="G148" t="n">
         <v>0</v>
       </c>
-      <c r="J148" t="inlineStr">
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1554996638- Nathalia Kodama Martins.zip</t>
         </is>
@@ -5771,10 +6344,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F149" t="inlineStr"/>
       <c r="G149" t="n">
         <v>0</v>
       </c>
-      <c r="J149" t="inlineStr">
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1047690907- Eloá Lamin da Gama.zip</t>
         </is>
@@ -5806,10 +6383,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F150" t="inlineStr"/>
       <c r="G150" t="n">
         <v>0</v>
       </c>
-      <c r="J150" t="inlineStr">
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1048132046- Wellington Eleuterio Alves.zip</t>
         </is>
@@ -5841,10 +6422,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F151" t="inlineStr"/>
       <c r="G151" t="n">
         <v>0</v>
       </c>
-      <c r="J151" t="inlineStr">
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1054939318-Ana Clara Poltronieri Borges.zip</t>
         </is>
@@ -5876,10 +6461,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F152" t="inlineStr"/>
       <c r="G152" t="n">
         <v>0</v>
       </c>
-      <c r="J152" t="inlineStr">
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1572734090- Rafaela Mattos.zip</t>
         </is>
@@ -5911,10 +6500,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F153" t="inlineStr"/>
       <c r="G153" t="n">
         <v>0</v>
       </c>
-      <c r="J153" t="inlineStr">
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-163799095- Laís Azevedo Fialho.zip</t>
         </is>
@@ -5946,10 +6539,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F154" t="inlineStr"/>
       <c r="G154" t="n">
         <v>0</v>
       </c>
-      <c r="J154" t="inlineStr">
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-164568903- Victor Duarte Faria.zip</t>
         </is>
@@ -5981,10 +6578,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F155" t="inlineStr"/>
       <c r="G155" t="n">
         <v>0</v>
       </c>
-      <c r="J155" t="inlineStr">
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-166019082- Karenn Andressa de Andrade Ticianel.zip</t>
         </is>
@@ -6016,10 +6617,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F156" t="inlineStr"/>
       <c r="G156" t="n">
         <v>0</v>
       </c>
-      <c r="J156" t="inlineStr">
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1667324052-ANDRESSA VITORINHO CERQUEIRA.zip</t>
         </is>
@@ -6051,10 +6656,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F157" t="inlineStr"/>
       <c r="G157" t="n">
         <v>0</v>
       </c>
-      <c r="J157" t="inlineStr">
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1699897241- Eloise Franciane Jardim Francisco.zip</t>
         </is>
@@ -6086,10 +6695,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F158" t="inlineStr"/>
       <c r="G158" t="n">
         <v>0</v>
       </c>
-      <c r="J158" t="inlineStr">
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1734293860- Gabriela Pereira Fregoneis.zip</t>
         </is>
@@ -6121,10 +6734,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F159" t="inlineStr"/>
       <c r="G159" t="n">
         <v>0</v>
       </c>
-      <c r="J159" t="inlineStr">
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1745253933- Eloá Lamin da Gama.zip</t>
         </is>
@@ -6156,10 +6773,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F160" t="inlineStr"/>
       <c r="G160" t="n">
         <v>0</v>
       </c>
-      <c r="J160" t="inlineStr">
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1766923734-Cairan Fagundes Jacintho.zip</t>
         </is>
@@ -6191,10 +6812,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F161" t="inlineStr"/>
       <c r="G161" t="n">
         <v>0</v>
       </c>
-      <c r="J161" t="inlineStr">
+      <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1795228596- O ARK.zip</t>
         </is>
@@ -6226,10 +6851,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F162" t="inlineStr"/>
       <c r="G162" t="n">
         <v>0</v>
       </c>
-      <c r="J162" t="inlineStr">
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1842378457- Kênia Bergo.zip</t>
         </is>
@@ -6261,10 +6890,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F163" t="inlineStr"/>
       <c r="G163" t="n">
         <v>0</v>
       </c>
-      <c r="J163" t="inlineStr">
+      <c r="H163" t="inlineStr"/>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-186654630- Thayse Maria Pires Fernandes.zip</t>
         </is>
@@ -6296,10 +6929,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F164" t="inlineStr"/>
       <c r="G164" t="n">
         <v>0</v>
       </c>
-      <c r="J164" t="inlineStr">
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-187238785- Juliano Ferreira.zip</t>
         </is>
@@ -6331,10 +6968,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F165" t="inlineStr"/>
       <c r="G165" t="n">
         <v>0</v>
       </c>
-      <c r="J165" t="inlineStr">
+      <c r="H165" t="inlineStr"/>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1314748063- Rebeca Marques.zip</t>
         </is>
@@ -6366,10 +7007,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F166" t="inlineStr"/>
       <c r="G166" t="n">
         <v>0</v>
       </c>
-      <c r="J166" t="inlineStr">
+      <c r="H166" t="inlineStr"/>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-132715746- Lissandra Felipe da Silva.zip</t>
         </is>
@@ -6401,10 +7046,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F167" t="inlineStr"/>
       <c r="G167" t="n">
         <v>0</v>
       </c>
-      <c r="J167" t="inlineStr">
+      <c r="H167" t="inlineStr"/>
+      <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1336109402-Andressa Vitorinho Cerqueira.zip</t>
         </is>
@@ -6436,10 +7085,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F168" t="inlineStr"/>
       <c r="G168" t="n">
         <v>0</v>
       </c>
-      <c r="J168" t="inlineStr">
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1922976160- Pedro Marques.zip</t>
         </is>
@@ -6471,10 +7124,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F169" t="inlineStr"/>
       <c r="G169" t="n">
         <v>0</v>
       </c>
-      <c r="J169" t="inlineStr">
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-193945435- Andressa Pamela de Oliveira.zip</t>
         </is>
@@ -6506,10 +7163,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F170" t="inlineStr"/>
       <c r="G170" t="n">
         <v>0</v>
       </c>
-      <c r="J170" t="inlineStr">
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1943667496-Lirian Lopes.zip</t>
         </is>
@@ -6541,10 +7202,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F171" t="inlineStr"/>
       <c r="G171" t="n">
         <v>0</v>
       </c>
-      <c r="J171" t="inlineStr">
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1987465659- Thiago Caleffi.zip</t>
         </is>
@@ -6576,10 +7241,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F172" t="inlineStr"/>
       <c r="G172" t="n">
         <v>0</v>
       </c>
-      <c r="J172" t="inlineStr">
+      <c r="H172" t="inlineStr"/>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1991836707-Bianca Beraldo.zip</t>
         </is>
@@ -6611,10 +7280,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F173" t="inlineStr"/>
       <c r="G173" t="n">
         <v>0</v>
       </c>
-      <c r="J173" t="inlineStr">
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2045187134- Gusta Valim Rossi.zip</t>
         </is>
@@ -6646,10 +7319,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F174" t="inlineStr"/>
       <c r="G174" t="n">
         <v>0</v>
       </c>
-      <c r="J174" t="inlineStr">
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2057203718-Leonardo Naves Cocco Pereira.zip</t>
         </is>
@@ -6681,10 +7358,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F175" t="inlineStr"/>
       <c r="G175" t="n">
         <v>0</v>
       </c>
-      <c r="J175" t="inlineStr">
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2068408980- Sandro Maranho Jacintho.zip</t>
         </is>
@@ -6716,10 +7397,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F176" t="inlineStr"/>
       <c r="G176" t="n">
         <v>0</v>
       </c>
-      <c r="J176" t="inlineStr">
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-20736232- Marcelo Yukio Goto.zip</t>
         </is>
@@ -6751,10 +7436,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F177" t="inlineStr"/>
       <c r="G177" t="n">
         <v>0</v>
       </c>
-      <c r="J177" t="inlineStr">
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2085118470- Gabriela Narumi Inoue.zip</t>
         </is>
@@ -6786,10 +7475,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F178" t="inlineStr"/>
       <c r="G178" t="n">
         <v>0</v>
       </c>
-      <c r="J178" t="inlineStr">
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2109546643- William Robson Cazavechia.zip</t>
         </is>
@@ -6821,10 +7514,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F179" t="inlineStr"/>
       <c r="G179" t="n">
         <v>0</v>
       </c>
-      <c r="J179" t="inlineStr">
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2122657518- Mariê.zip</t>
         </is>
@@ -6856,10 +7553,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F180" t="inlineStr"/>
       <c r="G180" t="n">
         <v>0</v>
       </c>
-      <c r="J180" t="inlineStr">
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2124685735-Lucas Fiorindo.zip</t>
         </is>
@@ -6891,10 +7592,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" t="n">
         <v>0</v>
       </c>
-      <c r="J181" t="inlineStr">
+      <c r="H181" t="inlineStr"/>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1555647500- sheliza onohine.zip</t>
         </is>
@@ -6926,10 +7631,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F182" t="inlineStr"/>
       <c r="G182" t="n">
         <v>0</v>
       </c>
-      <c r="J182" t="inlineStr">
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr"/>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1560371501- Rachel Coelho.zip</t>
         </is>
@@ -6961,10 +7670,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F183" t="inlineStr"/>
       <c r="G183" t="n">
         <v>0</v>
       </c>
-      <c r="J183" t="inlineStr">
+      <c r="H183" t="inlineStr"/>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1564768134-CANDELABRO PRODUÇÃO CÊNICA LTDA.zip</t>
         </is>
@@ -6996,10 +7709,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F184" t="inlineStr"/>
       <c r="G184" t="n">
         <v>0</v>
       </c>
-      <c r="J184" t="inlineStr">
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-22285065- Maria Gabre.zip</t>
         </is>
@@ -7031,10 +7748,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F185" t="inlineStr"/>
       <c r="G185" t="n">
         <v>0</v>
       </c>
-      <c r="J185" t="inlineStr">
+      <c r="H185" t="inlineStr"/>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-227680543- Matheus Gualda.zip</t>
         </is>
@@ -7066,10 +7787,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F186" t="inlineStr"/>
       <c r="G186" t="n">
         <v>0</v>
       </c>
-      <c r="J186" t="inlineStr">
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-229532248-RAFAEL OCHOA.zip</t>
         </is>
@@ -7101,10 +7826,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F187" t="inlineStr"/>
       <c r="G187" t="n">
         <v>0</v>
       </c>
-      <c r="J187" t="inlineStr">
+      <c r="H187" t="inlineStr"/>
+      <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-263527409- Joice Bianca Gomes.zip</t>
         </is>
@@ -7136,10 +7865,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F188" t="inlineStr"/>
       <c r="G188" t="n">
         <v>0</v>
       </c>
-      <c r="J188" t="inlineStr">
+      <c r="H188" t="inlineStr"/>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-28313918- Tauan Gonzalez Sposito.zip</t>
         </is>
@@ -7171,10 +7904,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F189" t="inlineStr"/>
       <c r="G189" t="n">
         <v>0</v>
       </c>
-      <c r="J189" t="inlineStr">
+      <c r="H189" t="inlineStr"/>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-399460469- Isadora Yalodê.zip</t>
         </is>
@@ -7206,10 +7943,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F190" t="inlineStr"/>
       <c r="G190" t="n">
         <v>0</v>
       </c>
-      <c r="J190" t="inlineStr">
+      <c r="H190" t="inlineStr"/>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-400977301- Ana Favorin.zip</t>
         </is>
@@ -7241,10 +7982,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F191" t="inlineStr"/>
       <c r="G191" t="n">
         <v>0</v>
       </c>
-      <c r="J191" t="inlineStr">
+      <c r="H191" t="inlineStr"/>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-419898531- Fernanda Inocente.zip</t>
         </is>
@@ -7276,10 +8021,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F192" t="inlineStr"/>
       <c r="G192" t="n">
         <v>0</v>
       </c>
-      <c r="J192" t="inlineStr">
+      <c r="H192" t="inlineStr"/>
+      <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-430119891- Ludmila de Almeida Castanheira.zip</t>
         </is>
@@ -7311,10 +8060,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F193" t="inlineStr"/>
       <c r="G193" t="n">
         <v>0</v>
       </c>
-      <c r="J193" t="inlineStr">
+      <c r="H193" t="inlineStr"/>
+      <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-441137618- Soraya Ayumi Tory.zip</t>
         </is>
@@ -7346,10 +8099,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F194" t="inlineStr"/>
       <c r="G194" t="n">
         <v>0</v>
       </c>
-      <c r="J194" t="inlineStr">
+      <c r="H194" t="inlineStr"/>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-44322422- Raquel Caroline Carreira Costa.zip</t>
         </is>
@@ -7381,10 +8138,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F195" t="inlineStr"/>
       <c r="G195" t="n">
         <v>0</v>
       </c>
-      <c r="J195" t="inlineStr">
+      <c r="H195" t="inlineStr"/>
+      <c r="I195" t="inlineStr"/>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-454118166- Felipe Index.zip</t>
         </is>
@@ -7416,10 +8177,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F196" t="inlineStr"/>
       <c r="G196" t="n">
         <v>0</v>
       </c>
-      <c r="J196" t="inlineStr">
+      <c r="H196" t="inlineStr"/>
+      <c r="I196" t="inlineStr"/>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-458896321- Jose Padilha.zip</t>
         </is>
@@ -7451,10 +8216,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F197" t="inlineStr"/>
       <c r="G197" t="n">
         <v>0</v>
       </c>
-      <c r="J197" t="inlineStr">
+      <c r="H197" t="inlineStr"/>
+      <c r="I197" t="inlineStr"/>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-459373355- Nayara Araujo.zip</t>
         </is>
@@ -7486,10 +8255,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F198" t="inlineStr"/>
       <c r="G198" t="n">
         <v>0</v>
       </c>
-      <c r="J198" t="inlineStr">
+      <c r="H198" t="inlineStr"/>
+      <c r="I198" t="inlineStr"/>
+      <c r="J198" t="inlineStr"/>
+      <c r="K198" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1874820470- roberta stubs parpinelli.zip</t>
         </is>
@@ -7521,10 +8294,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F199" t="inlineStr"/>
       <c r="G199" t="n">
         <v>0</v>
       </c>
-      <c r="J199" t="inlineStr">
+      <c r="H199" t="inlineStr"/>
+      <c r="I199" t="inlineStr"/>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-1904358682- Bárbara Bittencourt.zip</t>
         </is>
@@ -7556,10 +8333,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F200" t="inlineStr"/>
       <c r="G200" t="n">
         <v>0</v>
       </c>
-      <c r="J200" t="inlineStr">
+      <c r="H200" t="inlineStr"/>
+      <c r="I200" t="inlineStr"/>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-535569393-Raquel Caroline Carreira Costa.zip</t>
         </is>
@@ -7591,10 +8372,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F201" t="inlineStr"/>
       <c r="G201" t="n">
         <v>0</v>
       </c>
-      <c r="J201" t="inlineStr">
+      <c r="H201" t="inlineStr"/>
+      <c r="I201" t="inlineStr"/>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-539566482-Patrícia Dena Guimarães.zip</t>
         </is>
@@ -7626,10 +8411,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F202" t="inlineStr"/>
       <c r="G202" t="n">
         <v>0</v>
       </c>
-      <c r="J202" t="inlineStr">
+      <c r="H202" t="inlineStr"/>
+      <c r="I202" t="inlineStr"/>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-551187740-JONNATHAN RAMOS BATISTA.zip</t>
         </is>
@@ -7661,10 +8450,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F203" t="inlineStr"/>
       <c r="G203" t="n">
         <v>0</v>
       </c>
-      <c r="J203" t="inlineStr">
+      <c r="H203" t="inlineStr"/>
+      <c r="I203" t="inlineStr"/>
+      <c r="J203" t="inlineStr"/>
+      <c r="K203" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-567101368- William Farias.zip</t>
         </is>
@@ -7696,10 +8489,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F204" t="inlineStr"/>
       <c r="G204" t="n">
         <v>0</v>
       </c>
-      <c r="J204" t="inlineStr">
+      <c r="H204" t="inlineStr"/>
+      <c r="I204" t="inlineStr"/>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-569115175- André  Miranda.zip</t>
         </is>
@@ -7731,10 +8528,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F205" t="inlineStr"/>
       <c r="G205" t="n">
         <v>0</v>
       </c>
-      <c r="J205" t="inlineStr">
+      <c r="H205" t="inlineStr"/>
+      <c r="I205" t="inlineStr"/>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-57284498- Felipe Franco Tomazella.zip</t>
         </is>
@@ -7766,10 +8567,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F206" t="inlineStr"/>
       <c r="G206" t="n">
         <v>0</v>
       </c>
-      <c r="J206" t="inlineStr">
+      <c r="H206" t="inlineStr"/>
+      <c r="I206" t="inlineStr"/>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-574763939- José Carlos Leonel.zip</t>
         </is>
@@ -7801,10 +8606,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F207" t="inlineStr"/>
       <c r="G207" t="n">
         <v>0</v>
       </c>
-      <c r="J207" t="inlineStr">
+      <c r="H207" t="inlineStr"/>
+      <c r="I207" t="inlineStr"/>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-598560010- Vitoria Campanari.zip</t>
         </is>
@@ -7836,10 +8645,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F208" t="inlineStr"/>
       <c r="G208" t="n">
         <v>0</v>
       </c>
-      <c r="J208" t="inlineStr">
+      <c r="H208" t="inlineStr"/>
+      <c r="I208" t="inlineStr"/>
+      <c r="J208" t="inlineStr"/>
+      <c r="K208" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-621875312- Josimara de Oliveira Guerreiro.zip</t>
         </is>
@@ -7871,10 +8684,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F209" t="inlineStr"/>
       <c r="G209" t="n">
         <v>0</v>
       </c>
-      <c r="J209" t="inlineStr">
+      <c r="H209" t="inlineStr"/>
+      <c r="I209" t="inlineStr"/>
+      <c r="J209" t="inlineStr"/>
+      <c r="K209" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-642545826- Douglas Kodi Seto Takeguma.zip</t>
         </is>
@@ -7906,10 +8723,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F210" t="inlineStr"/>
       <c r="G210" t="n">
         <v>0</v>
       </c>
-      <c r="J210" t="inlineStr">
+      <c r="H210" t="inlineStr"/>
+      <c r="I210" t="inlineStr"/>
+      <c r="J210" t="inlineStr"/>
+      <c r="K210" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-677070345- André  Miranda.zip</t>
         </is>
@@ -7941,10 +8762,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F211" t="inlineStr"/>
       <c r="G211" t="n">
         <v>0</v>
       </c>
-      <c r="J211" t="inlineStr">
+      <c r="H211" t="inlineStr"/>
+      <c r="I211" t="inlineStr"/>
+      <c r="J211" t="inlineStr"/>
+      <c r="K211" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-727997397- Marcio Alex Pereira.zip</t>
         </is>
@@ -7976,10 +8801,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F212" t="inlineStr"/>
       <c r="G212" t="n">
         <v>0</v>
       </c>
-      <c r="J212" t="inlineStr">
+      <c r="H212" t="inlineStr"/>
+      <c r="I212" t="inlineStr"/>
+      <c r="J212" t="inlineStr"/>
+      <c r="K212" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-732850362- MARLI APARECIDA LEITE DA SILVA.zip</t>
         </is>
@@ -8011,10 +8840,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F213" t="inlineStr"/>
       <c r="G213" t="n">
         <v>0</v>
       </c>
-      <c r="J213" t="inlineStr">
+      <c r="H213" t="inlineStr"/>
+      <c r="I213" t="inlineStr"/>
+      <c r="J213" t="inlineStr"/>
+      <c r="K213" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-73364038-PATRÍCIA DENA GUIMARÃES.zip</t>
         </is>
@@ -8046,10 +8879,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F214" t="inlineStr"/>
       <c r="G214" t="n">
         <v>0</v>
       </c>
-      <c r="J214" t="inlineStr">
+      <c r="H214" t="inlineStr"/>
+      <c r="I214" t="inlineStr"/>
+      <c r="J214" t="inlineStr"/>
+      <c r="K214" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-761659965- Michelle Cerqueira César Tambosi.zip</t>
         </is>
@@ -8081,10 +8918,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F215" t="inlineStr"/>
       <c r="G215" t="n">
         <v>0</v>
       </c>
-      <c r="J215" t="inlineStr">
+      <c r="H215" t="inlineStr"/>
+      <c r="I215" t="inlineStr"/>
+      <c r="J215" t="inlineStr"/>
+      <c r="K215" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-2130849115- Mauro de Oliveira Junior.zip</t>
         </is>
@@ -8116,10 +8957,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F216" t="inlineStr"/>
       <c r="G216" t="n">
         <v>0</v>
       </c>
-      <c r="J216" t="inlineStr">
+      <c r="H216" t="inlineStr"/>
+      <c r="I216" t="inlineStr"/>
+      <c r="J216" t="inlineStr"/>
+      <c r="K216" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-80814193 - Rachel Coelho.zip</t>
         </is>
@@ -8151,10 +8996,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F217" t="inlineStr"/>
       <c r="G217" t="n">
         <v>0</v>
       </c>
-      <c r="J217" t="inlineStr">
+      <c r="H217" t="inlineStr"/>
+      <c r="I217" t="inlineStr"/>
+      <c r="J217" t="inlineStr"/>
+      <c r="K217" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-831663663- Lirian Lopes.zip</t>
         </is>
@@ -8186,10 +9035,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F218" t="inlineStr"/>
       <c r="G218" t="n">
         <v>0</v>
       </c>
-      <c r="J218" t="inlineStr">
+      <c r="H218" t="inlineStr"/>
+      <c r="I218" t="inlineStr"/>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-832658163- Ana Favorin.zip</t>
         </is>
@@ -8221,10 +9074,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F219" t="inlineStr"/>
       <c r="G219" t="n">
         <v>0</v>
       </c>
-      <c r="J219" t="inlineStr">
+      <c r="H219" t="inlineStr"/>
+      <c r="I219" t="inlineStr"/>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-833387025- Felipe de Moraes (Momo).zip</t>
         </is>
@@ -8256,10 +9113,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F220" t="inlineStr"/>
       <c r="G220" t="n">
         <v>0</v>
       </c>
-      <c r="J220" t="inlineStr">
+      <c r="H220" t="inlineStr"/>
+      <c r="I220" t="inlineStr"/>
+      <c r="J220" t="inlineStr"/>
+      <c r="K220" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-868895712-Fernando.zip</t>
         </is>
@@ -8291,10 +9152,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F221" t="inlineStr"/>
       <c r="G221" t="n">
         <v>0</v>
       </c>
-      <c r="J221" t="inlineStr">
+      <c r="H221" t="inlineStr"/>
+      <c r="I221" t="inlineStr"/>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-876163073- Carla Guizelini.zip</t>
         </is>
@@ -8326,10 +9191,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F222" t="inlineStr"/>
       <c r="G222" t="n">
         <v>0</v>
       </c>
-      <c r="J222" t="inlineStr">
+      <c r="H222" t="inlineStr"/>
+      <c r="I222" t="inlineStr"/>
+      <c r="J222" t="inlineStr"/>
+      <c r="K222" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-928980059- Beatriz Carrocini Colnago.zip</t>
         </is>
@@ -8361,10 +9230,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F223" t="inlineStr"/>
       <c r="G223" t="n">
         <v>0</v>
       </c>
-      <c r="J223" t="inlineStr">
+      <c r="H223" t="inlineStr"/>
+      <c r="I223" t="inlineStr"/>
+      <c r="J223" t="inlineStr"/>
+      <c r="K223" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-935028481- Giulia Cordeiro Faria.zip</t>
         </is>
@@ -8396,10 +9269,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F224" t="inlineStr"/>
       <c r="G224" t="n">
         <v>0</v>
       </c>
-      <c r="J224" t="inlineStr">
+      <c r="H224" t="inlineStr"/>
+      <c r="I224" t="inlineStr"/>
+      <c r="J224" t="inlineStr"/>
+      <c r="K224" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-9528432- Oni Kuroi.zip</t>
         </is>
@@ -8431,10 +9308,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F225" t="inlineStr"/>
       <c r="G225" t="n">
         <v>0</v>
       </c>
-      <c r="J225" t="inlineStr">
+      <c r="H225" t="inlineStr"/>
+      <c r="I225" t="inlineStr"/>
+      <c r="J225" t="inlineStr"/>
+      <c r="K225" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-958474622- Solange de Lima Munhoz.zip</t>
         </is>
@@ -8466,10 +9347,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F226" t="inlineStr"/>
       <c r="G226" t="n">
         <v>0</v>
       </c>
-      <c r="J226" t="inlineStr">
+      <c r="H226" t="inlineStr"/>
+      <c r="I226" t="inlineStr"/>
+      <c r="J226" t="inlineStr"/>
+      <c r="K226" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-962808927- Raquel Menegazzo.zip</t>
         </is>
@@ -8501,10 +9386,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F227" t="inlineStr"/>
       <c r="G227" t="n">
         <v>0</v>
       </c>
-      <c r="J227" t="inlineStr">
+      <c r="H227" t="inlineStr"/>
+      <c r="I227" t="inlineStr"/>
+      <c r="J227" t="inlineStr"/>
+      <c r="K227" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Oni Kuroi - on-246300286.zip</t>
         </is>
@@ -8536,10 +9425,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F228" t="inlineStr"/>
       <c r="G228" t="n">
         <v>0</v>
       </c>
-      <c r="J228" t="inlineStr">
+      <c r="H228" t="inlineStr"/>
+      <c r="I228" t="inlineStr"/>
+      <c r="J228" t="inlineStr"/>
+      <c r="K228" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer - PL - 16298-2022 - Sindicato Rural.txt</t>
         </is>
@@ -8571,10 +9464,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F229" t="inlineStr"/>
       <c r="G229" t="n">
         <v>0</v>
       </c>
-      <c r="J229" t="inlineStr">
+      <c r="H229" t="inlineStr"/>
+      <c r="I229" t="inlineStr"/>
+      <c r="J229" t="inlineStr"/>
+      <c r="K229" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer 64414_2021 PL 15996_2021 - fundo de vale.txt</t>
         </is>
@@ -8606,10 +9503,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F230" t="inlineStr"/>
       <c r="G230" t="n">
         <v>0</v>
       </c>
-      <c r="J230" t="inlineStr">
+      <c r="H230" t="inlineStr"/>
+      <c r="I230" t="inlineStr"/>
+      <c r="J230" t="inlineStr"/>
+      <c r="K230" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer 65391 2021 PL 15922 2021 CT Poluição.txt</t>
         </is>
@@ -8641,10 +9542,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F231" t="inlineStr"/>
       <c r="G231" t="n">
         <v>0</v>
       </c>
-      <c r="J231" t="inlineStr">
+      <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr"/>
+      <c r="J231" t="inlineStr"/>
+      <c r="K231" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-509149721-Fernando Aparecido Ponce Ribeiro.zip</t>
         </is>
@@ -8676,10 +9581,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F232" t="inlineStr"/>
       <c r="G232" t="n">
         <v>0</v>
       </c>
-      <c r="J232" t="inlineStr">
+      <c r="H232" t="inlineStr"/>
+      <c r="I232" t="inlineStr"/>
+      <c r="J232" t="inlineStr"/>
+      <c r="K232" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer 73514_2021 PL 15915_2021.txt</t>
         </is>
@@ -8711,10 +9620,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F233" t="inlineStr"/>
       <c r="G233" t="n">
         <v>0</v>
       </c>
-      <c r="J233" t="inlineStr">
+      <c r="H233" t="inlineStr"/>
+      <c r="I233" t="inlineStr"/>
+      <c r="J233" t="inlineStr"/>
+      <c r="K233" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\PARECER PL 16132_2022 Altera a Lei 9748_2014 - Exec. Música ao vivo.txt</t>
         </is>
@@ -8746,10 +9659,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F234" t="inlineStr"/>
       <c r="G234" t="n">
         <v>0</v>
       </c>
-      <c r="J234" t="inlineStr">
+      <c r="H234" t="inlineStr"/>
+      <c r="I234" t="inlineStr"/>
+      <c r="J234" t="inlineStr"/>
+      <c r="K234" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer PL 16305_2022 - CT Legislação - Processo n. 21896-2022.txt</t>
         </is>
@@ -8781,10 +9698,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F235" t="inlineStr"/>
       <c r="G235" t="n">
         <v>0</v>
       </c>
-      <c r="J235" t="inlineStr">
+      <c r="H235" t="inlineStr"/>
+      <c r="I235" t="inlineStr"/>
+      <c r="J235" t="inlineStr"/>
+      <c r="K235" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\PARECER PL 16354_2022 - Fomento às açoes sustentáveis para 17_08 - MANINHO_2022_Inst.Cesumar.txt</t>
         </is>
@@ -8816,10 +9737,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F236" t="inlineStr"/>
       <c r="G236" t="n">
         <v>0</v>
       </c>
-      <c r="J236" t="inlineStr">
+      <c r="H236" t="inlineStr"/>
+      <c r="I236" t="inlineStr"/>
+      <c r="J236" t="inlineStr"/>
+      <c r="K236" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\PARECER PL 16605_2023 - IPTU Verde - CREA.txt</t>
         </is>
@@ -8851,10 +9776,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F237" t="inlineStr"/>
       <c r="G237" t="n">
         <v>0</v>
       </c>
-      <c r="J237" t="inlineStr">
+      <c r="H237" t="inlineStr"/>
+      <c r="I237" t="inlineStr"/>
+      <c r="J237" t="inlineStr"/>
+      <c r="K237" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer PL N. 16342-2022.txt</t>
         </is>
@@ -8886,10 +9815,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F238" t="inlineStr"/>
       <c r="G238" t="n">
         <v>0</v>
       </c>
-      <c r="J238" t="inlineStr">
+      <c r="H238" t="inlineStr"/>
+      <c r="I238" t="inlineStr"/>
+      <c r="J238" t="inlineStr"/>
+      <c r="K238" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer PL Nº 2138_2022 - Cooperativas.txt</t>
         </is>
@@ -8921,10 +9854,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F239" t="inlineStr"/>
       <c r="G239" t="n">
         <v>0</v>
       </c>
-      <c r="J239" t="inlineStr">
+      <c r="H239" t="inlineStr"/>
+      <c r="I239" t="inlineStr"/>
+      <c r="J239" t="inlineStr"/>
+      <c r="K239" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer PL nº 2166_2022.txt</t>
         </is>
@@ -8956,10 +9893,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F240" t="inlineStr"/>
       <c r="G240" t="n">
         <v>0</v>
       </c>
-      <c r="J240" t="inlineStr">
+      <c r="H240" t="inlineStr"/>
+      <c r="I240" t="inlineStr"/>
+      <c r="J240" t="inlineStr"/>
+      <c r="K240" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer Programa IPTU Verde.txt</t>
         </is>
@@ -8991,10 +9932,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F241" t="inlineStr"/>
       <c r="G241" t="n">
         <v>0</v>
       </c>
-      <c r="J241" t="inlineStr">
+      <c r="H241" t="inlineStr"/>
+      <c r="I241" t="inlineStr"/>
+      <c r="J241" t="inlineStr"/>
+      <c r="K241" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer Programa IPTU Verde_2.txt</t>
         </is>
@@ -9026,10 +9971,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F242" t="inlineStr"/>
       <c r="G242" t="n">
         <v>0</v>
       </c>
-      <c r="J242" t="inlineStr">
+      <c r="H242" t="inlineStr"/>
+      <c r="I242" t="inlineStr"/>
+      <c r="J242" t="inlineStr"/>
+      <c r="K242" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer representatividade CMM no Comdema.txt</t>
         </is>
@@ -9061,10 +10010,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F243" t="inlineStr"/>
       <c r="G243" t="n">
         <v>0</v>
       </c>
-      <c r="J243" t="inlineStr">
+      <c r="H243" t="inlineStr"/>
+      <c r="I243" t="inlineStr"/>
+      <c r="J243" t="inlineStr"/>
+      <c r="K243" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\PARECER Resolução 01 IAM.txt</t>
         </is>
@@ -9096,10 +10049,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F244" t="inlineStr"/>
       <c r="G244" t="n">
         <v>0</v>
       </c>
-      <c r="J244" t="inlineStr">
+      <c r="H244" t="inlineStr"/>
+      <c r="I244" t="inlineStr"/>
+      <c r="J244" t="inlineStr"/>
+      <c r="K244" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\PARECER Resolução IAM Nº 03 2022.txt</t>
         </is>
@@ -9131,10 +10088,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F245" t="inlineStr"/>
       <c r="G245" t="n">
         <v>0</v>
       </c>
-      <c r="J245" t="inlineStr">
+      <c r="H245" t="inlineStr"/>
+      <c r="I245" t="inlineStr"/>
+      <c r="J245" t="inlineStr"/>
+      <c r="K245" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer Resolução IAM Nº 04 2022.txt</t>
         </is>
@@ -9166,10 +10127,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F246" t="inlineStr"/>
       <c r="G246" t="n">
         <v>0</v>
       </c>
-      <c r="J246" t="inlineStr">
+      <c r="H246" t="inlineStr"/>
+      <c r="I246" t="inlineStr"/>
+      <c r="J246" t="inlineStr"/>
+      <c r="K246" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Pedro Lucas Moro - on-1377007165.zip</t>
         </is>
@@ -9201,10 +10166,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F247" t="inlineStr"/>
       <c r="G247" t="n">
         <v>0</v>
       </c>
-      <c r="J247" t="inlineStr">
+      <c r="H247" t="inlineStr"/>
+      <c r="I247" t="inlineStr"/>
+      <c r="J247" t="inlineStr"/>
+      <c r="K247" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\on-784030336- Renan Gustavo Parma dos Reis.zip</t>
         </is>
@@ -9236,10 +10205,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F248" t="inlineStr"/>
       <c r="G248" t="n">
         <v>0</v>
       </c>
-      <c r="J248" t="inlineStr">
+      <c r="H248" t="inlineStr"/>
+      <c r="I248" t="inlineStr"/>
+      <c r="J248" t="inlineStr"/>
+      <c r="K248" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\ANDRÉ LUIS ROSA.zip</t>
         </is>
@@ -9271,10 +10244,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F249" t="inlineStr"/>
       <c r="G249" t="n">
         <v>0</v>
       </c>
-      <c r="J249" t="inlineStr">
+      <c r="H249" t="inlineStr"/>
+      <c r="I249" t="inlineStr"/>
+      <c r="J249" t="inlineStr"/>
+      <c r="K249" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Perímetro Municipal (19_01_2026).zip</t>
         </is>
@@ -9306,10 +10283,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F250" t="inlineStr"/>
       <c r="G250" t="n">
         <v>0</v>
       </c>
-      <c r="J250" t="inlineStr">
+      <c r="H250" t="inlineStr"/>
+      <c r="I250" t="inlineStr"/>
+      <c r="J250" t="inlineStr"/>
+      <c r="K250" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Perímetro Urbano (19_01_2026).zip</t>
         </is>
@@ -9341,10 +10322,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F251" t="inlineStr"/>
       <c r="G251" t="n">
         <v>0</v>
       </c>
-      <c r="J251" t="inlineStr">
+      <c r="H251" t="inlineStr"/>
+      <c r="I251" t="inlineStr"/>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Piera Paula Schnaider do Nascimento - on-177557296.zip</t>
         </is>
@@ -9376,10 +10361,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F252" t="inlineStr"/>
       <c r="G252" t="n">
         <v>0</v>
       </c>
-      <c r="J252" t="inlineStr">
+      <c r="H252" t="inlineStr"/>
+      <c r="I252" t="inlineStr"/>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\PLANILHA CONTROLE ORÇAMENTÁRIO (EXCEL) - Baixar Arquivo.txt</t>
         </is>
@@ -9411,10 +10400,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F253" t="inlineStr"/>
       <c r="G253" t="n">
         <v>0</v>
       </c>
-      <c r="J253" t="inlineStr">
+      <c r="H253" t="inlineStr"/>
+      <c r="I253" t="inlineStr"/>
+      <c r="J253" t="inlineStr"/>
+      <c r="K253" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Planilha de acompanhamento UBS.txt</t>
         </is>
@@ -9446,10 +10439,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F254" t="inlineStr"/>
       <c r="G254" t="n">
         <v>0</v>
       </c>
-      <c r="J254" t="inlineStr">
+      <c r="H254" t="inlineStr"/>
+      <c r="I254" t="inlineStr"/>
+      <c r="J254" t="inlineStr"/>
+      <c r="K254" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Plano de ação.txt</t>
         </is>
@@ -9481,10 +10478,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F255" t="inlineStr"/>
       <c r="G255" t="n">
         <v>0</v>
       </c>
-      <c r="J255" t="inlineStr">
+      <c r="H255" t="inlineStr"/>
+      <c r="I255" t="inlineStr"/>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Prestação de contas - Aniceto Matti - Parte 1.zip</t>
         </is>
@@ -9516,10 +10517,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F256" t="inlineStr"/>
       <c r="G256" t="n">
         <v>0</v>
       </c>
-      <c r="J256" t="inlineStr">
+      <c r="H256" t="inlineStr"/>
+      <c r="I256" t="inlineStr"/>
+      <c r="J256" t="inlineStr"/>
+      <c r="K256" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Prestação de contas - Aniceto Matti - Parte 2.zip</t>
         </is>
@@ -9551,10 +10556,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F257" t="inlineStr"/>
       <c r="G257" t="n">
         <v>0</v>
       </c>
-      <c r="J257" t="inlineStr">
+      <c r="H257" t="inlineStr"/>
+      <c r="I257" t="inlineStr"/>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Prestação de contas - Aniceto Matti - Parte 3.zip</t>
         </is>
@@ -9586,10 +10595,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F258" t="inlineStr"/>
       <c r="G258" t="n">
         <v>0</v>
       </c>
-      <c r="J258" t="inlineStr">
+      <c r="H258" t="inlineStr"/>
+      <c r="I258" t="inlineStr"/>
+      <c r="J258" t="inlineStr"/>
+      <c r="K258" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Proposta de alteração da LC 1093_2022.txt</t>
         </is>
@@ -9621,10 +10634,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F259" t="inlineStr"/>
       <c r="G259" t="n">
         <v>0</v>
       </c>
-      <c r="J259" t="inlineStr">
+      <c r="H259" t="inlineStr"/>
+      <c r="I259" t="inlineStr"/>
+      <c r="J259" t="inlineStr"/>
+      <c r="K259" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Quadra (19_01_2026).zip</t>
         </is>
@@ -9656,10 +10673,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F260" t="inlineStr"/>
       <c r="G260" t="n">
         <v>0</v>
       </c>
-      <c r="J260" t="inlineStr">
+      <c r="H260" t="inlineStr"/>
+      <c r="I260" t="inlineStr"/>
+      <c r="J260" t="inlineStr"/>
+      <c r="K260" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\RAFAELY PARMA DOS REIS.zip</t>
         </is>
@@ -9691,10 +10712,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F261" t="inlineStr"/>
       <c r="G261" t="n">
         <v>0</v>
       </c>
-      <c r="J261" t="inlineStr">
+      <c r="H261" t="inlineStr"/>
+      <c r="I261" t="inlineStr"/>
+      <c r="J261" t="inlineStr"/>
+      <c r="K261" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Raony Robson Ruiz - on-767380211.zip</t>
         </is>
@@ -9726,10 +10751,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F262" t="inlineStr"/>
       <c r="G262" t="n">
         <v>0</v>
       </c>
-      <c r="J262" t="inlineStr">
+      <c r="H262" t="inlineStr"/>
+      <c r="I262" t="inlineStr"/>
+      <c r="J262" t="inlineStr"/>
+      <c r="K262" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Parecer 69866_2021 PL 1989_2020.txt</t>
         </is>
@@ -9761,10 +10790,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F263" t="inlineStr"/>
       <c r="G263" t="n">
         <v>0</v>
       </c>
-      <c r="J263" t="inlineStr">
+      <c r="H263" t="inlineStr"/>
+      <c r="I263" t="inlineStr"/>
+      <c r="J263" t="inlineStr"/>
+      <c r="K263" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Wellington Eleuterio Alves.zip</t>
         </is>
@@ -9796,10 +10829,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F264" t="inlineStr"/>
       <c r="G264" t="n">
         <v>0</v>
       </c>
-      <c r="J264" t="inlineStr">
+      <c r="H264" t="inlineStr"/>
+      <c r="I264" t="inlineStr"/>
+      <c r="J264" t="inlineStr"/>
+      <c r="K264" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Vanderlei Junior.zip</t>
         </is>
@@ -9831,10 +10868,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F265" t="inlineStr"/>
       <c r="G265" t="n">
         <v>0</v>
       </c>
-      <c r="J265" t="inlineStr">
+      <c r="H265" t="inlineStr"/>
+      <c r="I265" t="inlineStr"/>
+      <c r="J265" t="inlineStr"/>
+      <c r="K265" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Vanderlei Junior - on-288379149.zip</t>
         </is>
@@ -9866,10 +10907,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F266" t="inlineStr"/>
       <c r="G266" t="n">
         <v>0</v>
       </c>
-      <c r="J266" t="inlineStr">
+      <c r="H266" t="inlineStr"/>
+      <c r="I266" t="inlineStr"/>
+      <c r="J266" t="inlineStr"/>
+      <c r="K266" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\160425145050_modelo__acordo_de_responsabilidade__rivv0_docx.docx.txt</t>
         </is>
@@ -9901,10 +10946,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F267" t="inlineStr"/>
       <c r="G267" t="n">
         <v>0</v>
       </c>
-      <c r="J267" t="inlineStr">
+      <c r="H267" t="inlineStr"/>
+      <c r="I267" t="inlineStr"/>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\220623133448_anexo_i__termo_autodeclaratorio__pequeno_gerador__23012023_docx.docx.txt</t>
         </is>
@@ -9936,10 +10985,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F268" t="inlineStr"/>
       <c r="G268" t="n">
         <v>0</v>
       </c>
-      <c r="J268" t="inlineStr">
+      <c r="H268" t="inlineStr"/>
+      <c r="I268" t="inlineStr"/>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\3ebee69fa294.docx.txt</t>
         </is>
@@ -9971,10 +11024,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F269" t="inlineStr"/>
       <c r="G269" t="n">
         <v>0</v>
       </c>
-      <c r="J269" t="inlineStr">
+      <c r="H269" t="inlineStr"/>
+      <c r="I269" t="inlineStr"/>
+      <c r="J269" t="inlineStr"/>
+      <c r="K269" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\5564c199f0e2.docx.txt</t>
         </is>
@@ -10006,10 +11063,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F270" t="inlineStr"/>
       <c r="G270" t="n">
         <v>0</v>
       </c>
-      <c r="J270" t="inlineStr">
+      <c r="H270" t="inlineStr"/>
+      <c r="I270" t="inlineStr"/>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\63d6d8362c55.docx.txt</t>
         </is>
@@ -10041,10 +11102,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F271" t="inlineStr"/>
       <c r="G271" t="n">
         <v>0</v>
       </c>
-      <c r="J271" t="inlineStr">
+      <c r="H271" t="inlineStr"/>
+      <c r="I271" t="inlineStr"/>
+      <c r="J271" t="inlineStr"/>
+      <c r="K271" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Adriana Quintino Sanchez Palacio  Tozatti.zip</t>
         </is>
@@ -10076,10 +11141,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F272" t="inlineStr"/>
       <c r="G272" t="n">
         <v>0</v>
       </c>
-      <c r="J272" t="inlineStr">
+      <c r="H272" t="inlineStr"/>
+      <c r="I272" t="inlineStr"/>
+      <c r="J272" t="inlineStr"/>
+      <c r="K272" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Alan Gaitarosso - on-1448752657.zip</t>
         </is>
@@ -10111,10 +11180,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F273" t="inlineStr"/>
       <c r="G273" t="n">
         <v>0</v>
       </c>
-      <c r="J273" t="inlineStr">
+      <c r="H273" t="inlineStr"/>
+      <c r="I273" t="inlineStr"/>
+      <c r="J273" t="inlineStr"/>
+      <c r="K273" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Alexandre Penha - on-1061167636.zip</t>
         </is>
@@ -10146,10 +11219,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F274" t="inlineStr"/>
       <c r="G274" t="n">
         <v>0</v>
       </c>
-      <c r="J274" t="inlineStr">
+      <c r="H274" t="inlineStr"/>
+      <c r="I274" t="inlineStr"/>
+      <c r="J274" t="inlineStr"/>
+      <c r="K274" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Alexandre Penha.zip</t>
         </is>
@@ -10181,10 +11258,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F275" t="inlineStr"/>
       <c r="G275" t="n">
         <v>0</v>
       </c>
-      <c r="J275" t="inlineStr">
+      <c r="H275" t="inlineStr"/>
+      <c r="I275" t="inlineStr"/>
+      <c r="J275" t="inlineStr"/>
+      <c r="K275" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Aline Luppi Grossi - on-1994472693.zip</t>
         </is>
@@ -10216,10 +11297,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F276" t="inlineStr"/>
       <c r="G276" t="n">
         <v>0</v>
       </c>
-      <c r="J276" t="inlineStr">
+      <c r="H276" t="inlineStr"/>
+      <c r="I276" t="inlineStr"/>
+      <c r="J276" t="inlineStr"/>
+      <c r="K276" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Ana Clara Poltronieri Borges.zip</t>
         </is>
@@ -10251,10 +11336,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F277" t="inlineStr"/>
       <c r="G277" t="n">
         <v>0</v>
       </c>
-      <c r="J277" t="inlineStr">
+      <c r="H277" t="inlineStr"/>
+      <c r="I277" t="inlineStr"/>
+      <c r="J277" t="inlineStr"/>
+      <c r="K277" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\ANDRESSA VITORINHO CERQUEIRA.zip</t>
         </is>
@@ -10286,10 +11375,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F278" t="inlineStr"/>
       <c r="G278" t="n">
         <v>0</v>
       </c>
-      <c r="J278" t="inlineStr">
+      <c r="H278" t="inlineStr"/>
+      <c r="I278" t="inlineStr"/>
+      <c r="J278" t="inlineStr"/>
+      <c r="K278" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\André Cesar Furlaneto Sampaio - on-1004931406.zip</t>
         </is>
@@ -10321,10 +11414,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F279" t="inlineStr"/>
       <c r="G279" t="n">
         <v>0</v>
       </c>
-      <c r="J279" t="inlineStr">
+      <c r="H279" t="inlineStr"/>
+      <c r="I279" t="inlineStr"/>
+      <c r="J279" t="inlineStr"/>
+      <c r="K279" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\William Robson Cazavechia - on-159152989.zip</t>
         </is>
@@ -10356,10 +11453,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F280" t="inlineStr"/>
       <c r="G280" t="n">
         <v>0</v>
       </c>
-      <c r="J280" t="inlineStr">
+      <c r="H280" t="inlineStr"/>
+      <c r="I280" t="inlineStr"/>
+      <c r="J280" t="inlineStr"/>
+      <c r="K280" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Érica Paiva Rosa - on-1356955037.zip</t>
         </is>
@@ -10391,10 +11492,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F281" t="inlineStr"/>
       <c r="G281" t="n">
         <v>0</v>
       </c>
-      <c r="J281" t="inlineStr">
+      <c r="H281" t="inlineStr"/>
+      <c r="I281" t="inlineStr"/>
+      <c r="J281" t="inlineStr"/>
+      <c r="K281" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\050124163339_termoautodeclaratoriograndegerador_docx.docx.txt</t>
         </is>
@@ -10426,10 +11531,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F282" t="inlineStr"/>
       <c r="G282" t="n">
         <v>0</v>
       </c>
-      <c r="J282" t="inlineStr">
+      <c r="H282" t="inlineStr"/>
+      <c r="I282" t="inlineStr"/>
+      <c r="J282" t="inlineStr"/>
+      <c r="K282" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Tiago Silva.zip</t>
         </is>
@@ -10461,10 +11570,14 @@
           <t>SEM_ARQUIVOS_ELEGIVEIS</t>
         </is>
       </c>
+      <c r="F283" t="inlineStr"/>
       <c r="G283" t="n">
         <v>0</v>
       </c>
-      <c r="J283" t="inlineStr">
+      <c r="H283" t="inlineStr"/>
+      <c r="I283" t="inlineStr"/>
+      <c r="J283" t="inlineStr"/>
+      <c r="K283" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\Vinícius Alves de Araujo.zip</t>
         </is>
@@ -10496,10 +11609,14 @@
           <t>ERRO_LEITURA</t>
         </is>
       </c>
+      <c r="F284" t="inlineStr"/>
       <c r="G284" t="n">
         <v>0</v>
       </c>
-      <c r="J284" t="inlineStr">
+      <c r="H284" t="inlineStr"/>
+      <c r="I284" t="inlineStr"/>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\certificados_inmetro-20260514.zip</t>
         </is>
@@ -10531,10 +11648,14 @@
           <t>ERRO_LEITURA</t>
         </is>
       </c>
+      <c r="F285" t="inlineStr"/>
       <c r="G285" t="n">
         <v>0</v>
       </c>
-      <c r="J285" t="inlineStr">
+      <c r="H285" t="inlineStr"/>
+      <c r="I285" t="inlineStr"/>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr">
         <is>
           <t>resultados\maringa_oficial\downloads\PLANILHA PGRCC - GRANDE GERADOR.xls</t>
         </is>

</xml_diff>